<commit_message>
ADP pricing sheet: invoiced pricing, new clients at bottom, package and list columns
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HvXhTSq2hCmheT3mKtqmHP
</commit_message>
<xml_diff>
--- a/output/stephen/CBA_Innovative_Advisors_ADP_2026-09-24.xlsx
+++ b/output/stephen/CBA_Innovative_Advisors_ADP_2026-09-24.xlsx
@@ -7,8 +7,7 @@
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="New Clients" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Payroll Packages" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Payroll Packages" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -22,7 +21,7 @@
     <numFmt numFmtId="165" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="166" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -76,6 +75,10 @@
     </font>
     <font>
       <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="13"/>
     </font>
@@ -84,7 +87,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -104,12 +107,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C00000"/>
+        <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9D9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C00000"/>
       </patternFill>
     </fill>
   </fills>
@@ -170,7 +178,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -260,7 +268,12 @@
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="4" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="right"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
     <xf numFmtId="166" fontId="4" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="right"/>
       <protection locked="0" hidden="0"/>
@@ -272,7 +285,49 @@
     <xf numFmtId="166" fontId="4" fillId="0" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="1">
       <protection locked="0" hidden="0"/>
     </xf>
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="right"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="5" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="right"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="right"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="right"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="right"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -280,9 +335,8 @@
       <alignment horizontal="left"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -637,28 +691,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:S122"/>
+  <dimension ref="A2:T122"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="15.5703125" defaultRowHeight="15"/>
   <cols>
     <col width="14.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
     <col width="14.28515625" customWidth="1" min="2" max="4"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="36.140625" bestFit="1" customWidth="1" min="5" max="5"/>
     <col width="36.140625" customWidth="1" min="6" max="8"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
     <col width="14.28515625" bestFit="1" customWidth="1" min="9" max="9"/>
     <col width="14.28515625" customWidth="1" min="10" max="10"/>
     <col width="15" bestFit="1" customWidth="1" min="11" max="11"/>
     <col width="15" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="13" customWidth="1" min="14" max="14"/>
     <col width="15" customWidth="1" min="15" max="16"/>
-    <col width="13" customWidth="1" min="16" max="16"/>
     <col width="18" bestFit="1" customWidth="1" min="17" max="17"/>
     <col width="26" customWidth="1" min="18" max="18"/>
-    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="15" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="2" ht="74.45" customHeight="1">
@@ -754,6 +802,11 @@
       </c>
       <c r="S2" s="15" t="inlineStr">
         <is>
+          <t>ADP list per run</t>
+        </is>
+      </c>
+      <c r="T2" s="15" t="inlineStr">
+        <is>
           <t>Invoice on file</t>
         </is>
       </c>
@@ -809,19 +862,15 @@
         <v>26</v>
       </c>
       <c r="L3" s="20" t="n">
-        <v>100.15</v>
+        <v>78.56999999999999</v>
       </c>
       <c r="M3" s="20">
         <f>K3*L3</f>
         <v/>
       </c>
       <c r="N3" s="21" t="n"/>
-      <c r="O3" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="P3" s="22" t="n">
-        <v>200</v>
-      </c>
+      <c r="O3" s="22" t="n"/>
+      <c r="P3" s="22" t="n"/>
       <c r="Q3" s="23">
         <f>M3</f>
         <v/>
@@ -831,7 +880,10 @@
           <t>ADP Enhanced Payroll</t>
         </is>
       </c>
-      <c r="S3" s="25" t="inlineStr">
+      <c r="S3" s="25" t="n">
+        <v>100.15</v>
+      </c>
+      <c r="T3" s="26" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -888,19 +940,15 @@
         <v>12</v>
       </c>
       <c r="L4" s="20" t="n">
-        <v>125.95</v>
+        <v>71.92</v>
       </c>
       <c r="M4" s="20">
         <f>K4*L4</f>
         <v/>
       </c>
       <c r="N4" s="21" t="n"/>
-      <c r="O4" s="22" t="n">
-        <v>0.91</v>
-      </c>
-      <c r="P4" s="22" t="n">
-        <v>200</v>
-      </c>
+      <c r="O4" s="22" t="n"/>
+      <c r="P4" s="22" t="n"/>
       <c r="Q4" s="23">
         <f>M4</f>
         <v/>
@@ -910,7 +958,10 @@
           <t>ADP Enhanced Payroll</t>
         </is>
       </c>
-      <c r="S4" s="25" t="inlineStr">
+      <c r="S4" s="25" t="n">
+        <v>125.95</v>
+      </c>
+      <c r="T4" s="26" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -967,19 +1018,15 @@
         <v>12</v>
       </c>
       <c r="L5" s="20" t="n">
-        <v>125.95</v>
+        <v>58</v>
       </c>
       <c r="M5" s="20">
         <f>K5*L5</f>
         <v/>
       </c>
       <c r="N5" s="21" t="n"/>
-      <c r="O5" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="P5" s="22" t="n">
-        <v>100</v>
-      </c>
+      <c r="O5" s="22" t="n"/>
+      <c r="P5" s="22" t="n"/>
       <c r="Q5" s="23">
         <f>M5</f>
         <v/>
@@ -989,7 +1036,10 @@
           <t>ADP Enhanced Payroll</t>
         </is>
       </c>
-      <c r="S5" s="25" t="inlineStr">
+      <c r="S5" s="25" t="n">
+        <v>125.95</v>
+      </c>
+      <c r="T5" s="26" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1046,19 +1096,15 @@
         <v>52</v>
       </c>
       <c r="L6" s="20" t="n">
-        <v>64.5</v>
+        <v>59.5</v>
       </c>
       <c r="M6" s="20">
         <f>K6*L6</f>
         <v/>
       </c>
       <c r="N6" s="21" t="n"/>
-      <c r="O6" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="P6" s="22" t="n">
-        <v>200</v>
-      </c>
+      <c r="O6" s="22" t="n"/>
+      <c r="P6" s="22" t="n"/>
       <c r="Q6" s="23">
         <f>M6</f>
         <v/>
@@ -1068,7 +1114,10 @@
           <t>ADP Enhanced Payroll</t>
         </is>
       </c>
-      <c r="S6" s="25" t="inlineStr">
+      <c r="S6" s="25" t="n">
+        <v>64.5</v>
+      </c>
+      <c r="T6" s="26" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1124,34 +1173,29 @@
       <c r="K7" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="L7" s="26" t="n">
+      <c r="L7" s="27" t="n">
+        <v>129.78</v>
+      </c>
+      <c r="M7" s="28">
+        <f>K7*L7</f>
+        <v/>
+      </c>
+      <c r="N7" s="6" t="n"/>
+      <c r="O7" s="29" t="n"/>
+      <c r="P7" s="29" t="n"/>
+      <c r="Q7" s="30">
+        <f>M7</f>
+        <v/>
+      </c>
+      <c r="R7" s="15" t="inlineStr">
+        <is>
+          <t>ADP Enhanced Payroll</t>
+        </is>
+      </c>
+      <c r="S7" s="31" t="n">
         <v>125.95</v>
       </c>
-      <c r="M7" s="26">
-        <f>K7*L7</f>
-        <v/>
-      </c>
-      <c r="N7" s="6" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O7" s="27" t="n">
-        <v>831.21</v>
-      </c>
-      <c r="P7" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q7" s="28">
-        <f>M7</f>
-        <v/>
-      </c>
-      <c r="R7" s="15" t="inlineStr">
-        <is>
-          <t>ADP Enhanced Payroll</t>
-        </is>
-      </c>
-      <c r="S7" t="inlineStr">
+      <c r="T7" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -1207,30 +1251,29 @@
       <c r="K8" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="L8" s="26" t="n">
+      <c r="L8" s="27" t="n">
+        <v>154.1</v>
+      </c>
+      <c r="M8" s="28">
+        <f>K8*L8</f>
+        <v/>
+      </c>
+      <c r="N8" s="6" t="n"/>
+      <c r="O8" s="29" t="n"/>
+      <c r="P8" s="29" t="n"/>
+      <c r="Q8" s="30">
+        <f>M8</f>
+        <v/>
+      </c>
+      <c r="R8" s="15" t="inlineStr">
+        <is>
+          <t>ADP Enhanced Payroll</t>
+        </is>
+      </c>
+      <c r="S8" s="31" t="n">
         <v>102.75</v>
       </c>
-      <c r="M8" s="26">
-        <f>K8*L8</f>
-        <v/>
-      </c>
-      <c r="N8" s="6" t="n"/>
-      <c r="O8" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="P8" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q8" s="28">
-        <f>M8</f>
-        <v/>
-      </c>
-      <c r="R8" s="15" t="inlineStr">
-        <is>
-          <t>ADP Enhanced Payroll</t>
-        </is>
-      </c>
-      <c r="S8" t="inlineStr">
+      <c r="T8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -1286,34 +1329,33 @@
       <c r="K9" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="L9" s="26" t="n">
+      <c r="L9" s="28" t="n">
+        <v>101</v>
+      </c>
+      <c r="M9" s="28">
+        <f>K9*L9</f>
+        <v/>
+      </c>
+      <c r="N9" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O9" s="29" t="n"/>
+      <c r="P9" s="29" t="n"/>
+      <c r="Q9" s="30">
+        <f>M9</f>
+        <v/>
+      </c>
+      <c r="R9" s="15" t="inlineStr">
+        <is>
+          <t>ADP Enhanced Payroll</t>
+        </is>
+      </c>
+      <c r="S9" s="32" t="n">
         <v>125.95</v>
       </c>
-      <c r="M9" s="26">
-        <f>K9*L9</f>
-        <v/>
-      </c>
-      <c r="N9" s="6" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O9" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="P9" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q9" s="28">
-        <f>M9</f>
-        <v/>
-      </c>
-      <c r="R9" s="15" t="inlineStr">
-        <is>
-          <t>ADP Enhanced Payroll</t>
-        </is>
-      </c>
-      <c r="S9" t="inlineStr">
+      <c r="T9" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -1369,34 +1411,29 @@
       <c r="K10" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="L10" s="26" t="n">
+      <c r="L10" s="28" t="n">
+        <v>98.5</v>
+      </c>
+      <c r="M10" s="28">
+        <f>K10*L10</f>
+        <v/>
+      </c>
+      <c r="N10" s="6" t="n"/>
+      <c r="O10" s="29" t="n"/>
+      <c r="P10" s="29" t="n"/>
+      <c r="Q10" s="30">
+        <f>M10</f>
+        <v/>
+      </c>
+      <c r="R10" s="15" t="inlineStr">
+        <is>
+          <t>ADP Enhanced Payroll</t>
+        </is>
+      </c>
+      <c r="S10" s="32" t="n">
         <v>106.55</v>
       </c>
-      <c r="M10" s="26">
-        <f>K10*L10</f>
-        <v/>
-      </c>
-      <c r="N10" s="6" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O10" s="27" t="n">
-        <v>1308.24</v>
-      </c>
-      <c r="P10" s="27" t="n">
-        <v>200</v>
-      </c>
-      <c r="Q10" s="28">
-        <f>M10</f>
-        <v/>
-      </c>
-      <c r="R10" s="15" t="inlineStr">
-        <is>
-          <t>ADP Enhanced Payroll</t>
-        </is>
-      </c>
-      <c r="S10" t="inlineStr">
+      <c r="T10" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -1452,10 +1489,10 @@
       <c r="K11" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="L11" s="26" t="n">
+      <c r="L11" s="28" t="n">
         <v>261.95</v>
       </c>
-      <c r="M11" s="26">
+      <c r="M11" s="28">
         <f>K11*L11</f>
         <v/>
       </c>
@@ -1464,13 +1501,9 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="O11" s="27" t="n">
-        <v>812.8</v>
-      </c>
-      <c r="P11" s="27" t="n">
-        <v>100</v>
-      </c>
-      <c r="Q11" s="28">
+      <c r="O11" s="29" t="n"/>
+      <c r="P11" s="29" t="n"/>
+      <c r="Q11" s="30">
         <f>M11</f>
         <v/>
       </c>
@@ -1479,7 +1512,10 @@
           <t>ADP HR Pro</t>
         </is>
       </c>
-      <c r="S11" t="inlineStr">
+      <c r="S11" s="32" t="n">
+        <v>261.95</v>
+      </c>
+      <c r="T11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -1535,34 +1571,33 @@
       <c r="K12" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="L12" s="26" t="n">
+      <c r="L12" s="28" t="n">
+        <v>77</v>
+      </c>
+      <c r="M12" s="28">
+        <f>K12*L12</f>
+        <v/>
+      </c>
+      <c r="N12" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O12" s="29" t="n"/>
+      <c r="P12" s="29" t="n"/>
+      <c r="Q12" s="30">
+        <f>M12</f>
+        <v/>
+      </c>
+      <c r="R12" s="15" t="inlineStr">
+        <is>
+          <t>ADP Enhanced Payroll</t>
+        </is>
+      </c>
+      <c r="S12" s="32" t="n">
         <v>133.25</v>
       </c>
-      <c r="M12" s="26">
-        <f>K12*L12</f>
-        <v/>
-      </c>
-      <c r="N12" s="6" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O12" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="P12" s="27" t="n">
-        <v>100</v>
-      </c>
-      <c r="Q12" s="28">
-        <f>M12</f>
-        <v/>
-      </c>
-      <c r="R12" s="15" t="inlineStr">
-        <is>
-          <t>ADP Enhanced Payroll</t>
-        </is>
-      </c>
-      <c r="S12" t="inlineStr">
+      <c r="T12" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -1618,10 +1653,10 @@
       <c r="K13" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="L13" s="26" t="n">
-        <v>129.6</v>
-      </c>
-      <c r="M13" s="26">
+      <c r="L13" s="28" t="n">
+        <v>100</v>
+      </c>
+      <c r="M13" s="28">
         <f>K13*L13</f>
         <v/>
       </c>
@@ -1632,7 +1667,7 @@
       </c>
       <c r="O13" s="4" t="n"/>
       <c r="P13" s="4" t="n"/>
-      <c r="Q13" s="28">
+      <c r="Q13" s="30">
         <f>M13</f>
         <v/>
       </c>
@@ -1641,7 +1676,10 @@
           <t>ADP Enhanced Payroll</t>
         </is>
       </c>
-      <c r="S13" t="inlineStr">
+      <c r="S13" s="32" t="n">
+        <v>129.6</v>
+      </c>
+      <c r="T13" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -1663,7 +1701,7 @@
       </c>
       <c r="D14" s="1" t="inlineStr">
         <is>
-          <t>New/Gusto</t>
+          <t>Existing</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1697,10 +1735,10 @@
       <c r="K14" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="L14" s="26" t="n">
-        <v>125.95</v>
-      </c>
-      <c r="M14" s="26">
+      <c r="L14" s="28" t="n">
+        <v>50</v>
+      </c>
+      <c r="M14" s="28">
         <f>K14*L14</f>
         <v/>
       </c>
@@ -1711,7 +1749,7 @@
       </c>
       <c r="O14" s="4" t="n"/>
       <c r="P14" s="4" t="n"/>
-      <c r="Q14" s="28">
+      <c r="Q14" s="30">
         <f>M14</f>
         <v/>
       </c>
@@ -1720,7 +1758,10 @@
           <t>ADP Enhanced Payroll</t>
         </is>
       </c>
-      <c r="S14" t="inlineStr">
+      <c r="S14" s="32" t="n">
+        <v>125.95</v>
+      </c>
+      <c r="T14" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -1742,7 +1783,7 @@
       </c>
       <c r="D15" s="1" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Existing</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1776,10 +1817,10 @@
       <c r="K15" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="L15" s="26" t="n">
-        <v>500</v>
-      </c>
-      <c r="M15" s="26">
+      <c r="L15" s="28" t="n">
+        <v>400</v>
+      </c>
+      <c r="M15" s="28">
         <f>K15*L15</f>
         <v/>
       </c>
@@ -1790,7 +1831,7 @@
       </c>
       <c r="O15" s="4" t="n"/>
       <c r="P15" s="4" t="n"/>
-      <c r="Q15" s="28">
+      <c r="Q15" s="30">
         <f>M15</f>
         <v/>
       </c>
@@ -1799,156 +1840,72 @@
           <t>ADP Essential Payroll</t>
         </is>
       </c>
-      <c r="S15" t="inlineStr">
+      <c r="S15" s="32" t="n">
+        <v>500</v>
+      </c>
+      <c r="T15" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
-        <v>14</v>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Frank </t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Giordano </t>
-        </is>
-      </c>
-      <c r="D16" s="1" t="inlineStr">
-        <is>
-          <t>New/Gusto</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>FRG Advisory, LLC</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>40-0020506</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>431 E 20th Street</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>New York NY 10010</t>
-        </is>
-      </c>
-      <c r="I16" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J16" s="3" t="inlineStr">
-        <is>
-          <t>Monthly</t>
-        </is>
-      </c>
-      <c r="K16" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="L16" s="29" t="n">
-        <v>70</v>
-      </c>
-      <c r="M16" s="6">
-        <f>K16*L16</f>
-        <v/>
-      </c>
-      <c r="N16" s="6" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A16" s="1" t="n"/>
+      <c r="B16" s="2" t="n"/>
+      <c r="C16" s="2" t="n"/>
+      <c r="D16" s="1" t="n"/>
+      <c r="E16" s="2" t="n"/>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="n"/>
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="3" t="n"/>
+      <c r="J16" s="3" t="n"/>
+      <c r="K16" s="4" t="n"/>
+      <c r="L16" s="33" t="n"/>
+      <c r="M16" s="6" t="n"/>
+      <c r="N16" s="6" t="n"/>
       <c r="O16" s="4" t="n"/>
       <c r="P16" s="4" t="n"/>
       <c r="Q16" s="5" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
-        <v>15</v>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Alexander </t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Harris</t>
-        </is>
-      </c>
-      <c r="D17" s="1" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>Kapstone Digital LLC</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>85-3782692</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>936 SW 1st Ave Apt. No. 406</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>Miami, FL 33130</t>
-        </is>
-      </c>
-      <c r="I17" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J17" s="3" t="inlineStr">
-        <is>
-          <t>Monthly</t>
-        </is>
-      </c>
-      <c r="K17" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="L17" s="29" t="n">
-        <v>70</v>
-      </c>
-      <c r="M17" s="6">
-        <f>K17*L17</f>
-        <v/>
-      </c>
-      <c r="N17" s="6" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O17" s="4" t="n"/>
-      <c r="P17" s="4" t="n"/>
-      <c r="Q17" s="5" t="n"/>
+      <c r="A17" s="34" t="n"/>
+      <c r="B17" s="35" t="inlineStr">
+        <is>
+          <t>NEW CLIENTS</t>
+        </is>
+      </c>
+      <c r="C17" s="36" t="n"/>
+      <c r="D17" s="34" t="n"/>
+      <c r="E17" s="36" t="n"/>
+      <c r="F17" s="36" t="n"/>
+      <c r="G17" s="36" t="n"/>
+      <c r="H17" s="36" t="n"/>
+      <c r="I17" s="37" t="n"/>
+      <c r="J17" s="37" t="n"/>
+      <c r="K17" s="38" t="n"/>
+      <c r="L17" s="39" t="n"/>
+      <c r="M17" s="40" t="n"/>
+      <c r="N17" s="40" t="n"/>
+      <c r="O17" s="38" t="n"/>
+      <c r="P17" s="38" t="n"/>
+      <c r="Q17" s="41" t="n"/>
+      <c r="R17" s="42" t="n"/>
+      <c r="S17" s="42" t="n"/>
+      <c r="T17" s="42" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Benjamin</t>
+          <t>Oliver</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Solomon </t>
+          <t>Beirne</t>
         </is>
       </c>
       <c r="D18" s="1" t="inlineStr">
@@ -1958,39 +1915,39 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Broadway 2000, Inc</t>
+          <t>B333 Trading Group LLC</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>85-3662838</t>
+          <t>42-2175878</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>662 Driggs Avenue</t>
+          <t>980 N Federal Hwy Suite 314</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Brooklyn, NY 11211</t>
+          <t>Boca Raton FL 33432</t>
         </is>
       </c>
       <c r="I18" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>Yearly</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="K18" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L18" s="29" t="n">
-        <v>300</v>
-      </c>
-      <c r="M18" s="6">
+        <v>12</v>
+      </c>
+      <c r="L18" s="28" t="n">
+        <v>77</v>
+      </c>
+      <c r="M18" s="28">
         <f>K18*L18</f>
         <v/>
       </c>
@@ -2001,20 +1958,36 @@
       </c>
       <c r="O18" s="4" t="n"/>
       <c r="P18" s="4" t="n"/>
-      <c r="Q18" s="5" t="n"/>
+      <c r="Q18" s="30">
+        <f>M18</f>
+        <v/>
+      </c>
+      <c r="R18" s="15" t="inlineStr">
+        <is>
+          <t>ADP Enhanced Payroll</t>
+        </is>
+      </c>
+      <c r="S18" s="32" t="n">
+        <v>129.6</v>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>John</t>
+          <t xml:space="preserve">Anthony </t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Ewing</t>
+          <t xml:space="preserve">Gerb </t>
         </is>
       </c>
       <c r="D19" s="1" t="inlineStr">
@@ -2024,22 +1997,22 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Atlas Opera, Inc.</t>
+          <t>AJG Trading LLC</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>82-2302400</t>
+          <t>41-5035542</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>83 Canal Street</t>
+          <t>1881 N Nash Street Apt No 705</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>New York, NY 10002</t>
+          <t>Arlington, VA 22209</t>
         </is>
       </c>
       <c r="I19" s="3" t="n">
@@ -2053,30 +2026,50 @@
       <c r="K19" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="L19" s="29" t="n">
+      <c r="L19" s="28" t="n">
         <v>70</v>
       </c>
-      <c r="M19" s="6">
+      <c r="M19" s="28">
         <f>K19*L19</f>
         <v/>
       </c>
-      <c r="N19" s="6" t="n"/>
+      <c r="N19" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="O19" s="4" t="n"/>
       <c r="P19" s="4" t="n"/>
-      <c r="Q19" s="5" t="n"/>
+      <c r="Q19" s="30">
+        <f>M19</f>
+        <v/>
+      </c>
+      <c r="R19" s="15" t="inlineStr">
+        <is>
+          <t>ADP Enhanced Payroll</t>
+        </is>
+      </c>
+      <c r="S19" s="32" t="n">
+        <v>125.95</v>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Christina </t>
+          <t xml:space="preserve">Alexander </t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pellicane </t>
+          <t>Harris</t>
         </is>
       </c>
       <c r="D20" s="1" t="inlineStr">
@@ -2086,22 +2079,22 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>North Star Works, LLC</t>
+          <t>Kapstone Digital LLC</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>42-4495054</t>
+          <t>85-3782692</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>121 S Colts Neck Way</t>
+          <t>936 SW 1st Ave Apt. No. 406</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Hockessin, DE 19707</t>
+          <t>Miami, FL 33130</t>
         </is>
       </c>
       <c r="I20" s="3" t="n">
@@ -2115,10 +2108,10 @@
       <c r="K20" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="L20" s="29" t="n">
-        <v>50</v>
-      </c>
-      <c r="M20" s="6">
+      <c r="L20" s="28" t="n">
+        <v>70</v>
+      </c>
+      <c r="M20" s="28">
         <f>K20*L20</f>
         <v/>
       </c>
@@ -2129,49 +2122,183 @@
       </c>
       <c r="O20" s="4" t="n"/>
       <c r="P20" s="4" t="n"/>
-      <c r="Q20" s="5" t="n"/>
+      <c r="Q20" s="30">
+        <f>M20</f>
+        <v/>
+      </c>
+      <c r="R20" s="15" t="inlineStr">
+        <is>
+          <t>ADP Enhanced Payroll</t>
+        </is>
+      </c>
+      <c r="S20" s="32" t="n">
+        <v>125.95</v>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>19</v>
-      </c>
-      <c r="B21" s="2" t="n"/>
-      <c r="C21" s="2" t="n"/>
-      <c r="D21" s="1" t="n"/>
-      <c r="E21" s="2" t="n"/>
-      <c r="F21" s="2" t="n"/>
-      <c r="G21" s="2" t="n"/>
-      <c r="H21" s="2" t="n"/>
-      <c r="I21" s="3" t="n"/>
-      <c r="J21" s="3" t="n"/>
-      <c r="K21" s="4" t="n"/>
-      <c r="L21" s="29" t="n"/>
-      <c r="M21" s="6" t="n"/>
+        <v>17</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>John</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Ewing</t>
+        </is>
+      </c>
+      <c r="D21" s="1" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Atlas Opera, Inc.</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>82-2302400</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>83 Canal Street</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>New York, NY 10002</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="K21" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="L21" s="28" t="n">
+        <v>70</v>
+      </c>
+      <c r="M21" s="28">
+        <f>K21*L21</f>
+        <v/>
+      </c>
       <c r="N21" s="6" t="n"/>
       <c r="O21" s="4" t="n"/>
       <c r="P21" s="4" t="n"/>
-      <c r="Q21" s="5" t="n"/>
+      <c r="Q21" s="30">
+        <f>M21</f>
+        <v/>
+      </c>
+      <c r="R21" s="15" t="inlineStr">
+        <is>
+          <t>ADP Enhanced Payroll</t>
+        </is>
+      </c>
+      <c r="S21" s="32" t="n">
+        <v>125.95</v>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>20</v>
-      </c>
-      <c r="B22" s="2" t="n"/>
-      <c r="C22" s="2" t="n"/>
-      <c r="D22" s="1" t="n"/>
-      <c r="E22" s="2" t="n"/>
-      <c r="F22" s="2" t="n"/>
-      <c r="G22" s="2" t="n"/>
-      <c r="H22" s="2" t="n"/>
-      <c r="I22" s="3" t="n"/>
-      <c r="J22" s="3" t="n"/>
-      <c r="K22" s="4" t="n"/>
-      <c r="L22" s="29" t="n"/>
-      <c r="M22" s="6" t="n"/>
-      <c r="N22" s="6" t="n"/>
+        <v>18</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Christina </t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pellicane </t>
+        </is>
+      </c>
+      <c r="D22" s="1" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>North Star Works, LLC</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>42-4495054</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>121 S Colts Neck Way</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Hockessin, DE 19707</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="K22" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="L22" s="28" t="n">
+        <v>50</v>
+      </c>
+      <c r="M22" s="28">
+        <f>K22*L22</f>
+        <v/>
+      </c>
+      <c r="N22" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="O22" s="4" t="n"/>
       <c r="P22" s="4" t="n"/>
-      <c r="Q22" s="5" t="n"/>
+      <c r="Q22" s="30">
+        <f>M22</f>
+        <v/>
+      </c>
+      <c r="R22" s="15" t="inlineStr">
+        <is>
+          <t>ADP Enhanced Payroll</t>
+        </is>
+      </c>
+      <c r="S22" s="32" t="n">
+        <v>125.95</v>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
@@ -2187,8 +2314,15 @@
       <c r="I23" s="3" t="n"/>
       <c r="J23" s="3" t="n"/>
       <c r="K23" s="4" t="n"/>
-      <c r="L23" s="29" t="n"/>
-      <c r="M23" s="6" t="n"/>
+      <c r="L23" s="43" t="inlineStr">
+        <is>
+          <t>New clients total</t>
+        </is>
+      </c>
+      <c r="M23" s="44">
+        <f>SUM(M18:M22)</f>
+        <v/>
+      </c>
       <c r="N23" s="6" t="n"/>
       <c r="O23" s="4" t="n"/>
       <c r="P23" s="4" t="n"/>
@@ -2208,7 +2342,7 @@
       <c r="I24" s="3" t="n"/>
       <c r="J24" s="3" t="n"/>
       <c r="K24" s="4" t="n"/>
-      <c r="L24" s="29" t="n"/>
+      <c r="L24" s="33" t="n"/>
       <c r="M24" s="6" t="n"/>
       <c r="N24" s="6" t="n"/>
       <c r="O24" s="4" t="n"/>
@@ -2229,7 +2363,7 @@
       <c r="I25" s="3" t="n"/>
       <c r="J25" s="3" t="n"/>
       <c r="K25" s="4" t="n"/>
-      <c r="L25" s="29" t="n"/>
+      <c r="L25" s="33" t="n"/>
       <c r="M25" s="6" t="n"/>
       <c r="N25" s="6" t="n"/>
       <c r="O25" s="4" t="n"/>
@@ -2250,7 +2384,7 @@
       <c r="I26" s="3" t="n"/>
       <c r="J26" s="3" t="n"/>
       <c r="K26" s="4" t="n"/>
-      <c r="L26" s="29" t="n"/>
+      <c r="L26" s="33" t="n"/>
       <c r="M26" s="6" t="n"/>
       <c r="N26" s="6" t="n"/>
       <c r="O26" s="4" t="n"/>
@@ -2271,7 +2405,7 @@
       <c r="I27" s="3" t="n"/>
       <c r="J27" s="3" t="n"/>
       <c r="K27" s="4" t="n"/>
-      <c r="L27" s="29" t="n"/>
+      <c r="L27" s="33" t="n"/>
       <c r="M27" s="6" t="n"/>
       <c r="N27" s="6" t="n"/>
       <c r="O27" s="4" t="n"/>
@@ -2292,7 +2426,7 @@
       <c r="I28" s="3" t="n"/>
       <c r="J28" s="3" t="n"/>
       <c r="K28" s="4" t="n"/>
-      <c r="L28" s="29" t="n"/>
+      <c r="L28" s="33" t="n"/>
       <c r="M28" s="6" t="n"/>
       <c r="N28" s="6" t="n"/>
       <c r="O28" s="4" t="n"/>
@@ -2313,13 +2447,13 @@
       <c r="I29" s="3" t="n"/>
       <c r="J29" s="3" t="n"/>
       <c r="K29" s="4" t="n"/>
-      <c r="L29" s="30" t="inlineStr">
+      <c r="L29" s="45" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
       <c r="M29" s="12">
-        <f>SUM(M3:M26)</f>
+        <f>SUM(M3:M15)</f>
         <v/>
       </c>
       <c r="N29" s="6" t="n"/>
@@ -2341,7 +2475,7 @@
       <c r="I30" s="3" t="n"/>
       <c r="J30" s="3" t="n"/>
       <c r="K30" s="4" t="n"/>
-      <c r="L30" s="30" t="n"/>
+      <c r="L30" s="45" t="n"/>
       <c r="M30" s="11" t="n"/>
       <c r="N30" s="6" t="n"/>
       <c r="O30" s="4" t="n"/>
@@ -2362,7 +2496,7 @@
       <c r="I31" s="3" t="n"/>
       <c r="J31" s="3" t="n"/>
       <c r="K31" s="4" t="n"/>
-      <c r="L31" s="30" t="inlineStr">
+      <c r="L31" s="45" t="inlineStr">
         <is>
           <t>Multiplier</t>
         </is>
@@ -2390,7 +2524,7 @@
       <c r="I32" s="3" t="n"/>
       <c r="J32" s="3" t="n"/>
       <c r="K32" s="4" t="n"/>
-      <c r="L32" s="29" t="n"/>
+      <c r="L32" s="33" t="n"/>
       <c r="M32" s="11" t="n"/>
       <c r="N32" s="6" t="n"/>
       <c r="O32" s="4" t="n"/>
@@ -2411,7 +2545,7 @@
       <c r="I33" s="3" t="n"/>
       <c r="J33" s="3" t="n"/>
       <c r="K33" s="4" t="n"/>
-      <c r="L33" s="29" t="n"/>
+      <c r="L33" s="33" t="n"/>
       <c r="M33" s="6" t="n"/>
       <c r="N33" s="6" t="n"/>
       <c r="O33" s="4" t="n"/>
@@ -2432,7 +2566,7 @@
       <c r="I34" s="3" t="n"/>
       <c r="J34" s="3" t="n"/>
       <c r="K34" s="4" t="n"/>
-      <c r="L34" s="29" t="n"/>
+      <c r="L34" s="33" t="n"/>
       <c r="M34" s="6" t="n"/>
       <c r="N34" s="6" t="n"/>
       <c r="O34" s="4" t="n"/>
@@ -2453,7 +2587,7 @@
       <c r="I35" s="3" t="n"/>
       <c r="J35" s="3" t="n"/>
       <c r="K35" s="4" t="n"/>
-      <c r="L35" s="29" t="n"/>
+      <c r="L35" s="33" t="n"/>
       <c r="M35" s="6" t="n"/>
       <c r="N35" s="6" t="n"/>
       <c r="O35" s="4" t="n"/>
@@ -2474,7 +2608,7 @@
       <c r="I36" s="3" t="n"/>
       <c r="J36" s="3" t="n"/>
       <c r="K36" s="4" t="n"/>
-      <c r="L36" s="29" t="n"/>
+      <c r="L36" s="33" t="n"/>
       <c r="M36" s="6" t="n"/>
       <c r="N36" s="6" t="n"/>
       <c r="O36" s="4" t="n"/>
@@ -2495,7 +2629,7 @@
       <c r="I37" s="3" t="n"/>
       <c r="J37" s="3" t="n"/>
       <c r="K37" s="4" t="n"/>
-      <c r="L37" s="29" t="n"/>
+      <c r="L37" s="33" t="n"/>
       <c r="M37" s="6" t="n"/>
       <c r="N37" s="6" t="n"/>
       <c r="O37" s="4" t="n"/>
@@ -2516,7 +2650,7 @@
       <c r="I38" s="3" t="n"/>
       <c r="J38" s="3" t="n"/>
       <c r="K38" s="4" t="n"/>
-      <c r="L38" s="29" t="n"/>
+      <c r="L38" s="33" t="n"/>
       <c r="M38" s="6" t="n"/>
       <c r="N38" s="6" t="n"/>
       <c r="O38" s="4" t="n"/>
@@ -2537,7 +2671,7 @@
       <c r="I39" s="3" t="n"/>
       <c r="J39" s="3" t="n"/>
       <c r="K39" s="4" t="n"/>
-      <c r="L39" s="29" t="n"/>
+      <c r="L39" s="33" t="n"/>
       <c r="M39" s="6" t="n"/>
       <c r="N39" s="6" t="n"/>
       <c r="O39" s="4" t="n"/>
@@ -2558,7 +2692,7 @@
       <c r="I40" s="3" t="n"/>
       <c r="J40" s="3" t="n"/>
       <c r="K40" s="4" t="n"/>
-      <c r="L40" s="29" t="n"/>
+      <c r="L40" s="33" t="n"/>
       <c r="M40" s="6" t="n"/>
       <c r="N40" s="6" t="n"/>
       <c r="O40" s="4" t="n"/>
@@ -2579,7 +2713,7 @@
       <c r="I41" s="3" t="n"/>
       <c r="J41" s="3" t="n"/>
       <c r="K41" s="4" t="n"/>
-      <c r="L41" s="29" t="n"/>
+      <c r="L41" s="33" t="n"/>
       <c r="M41" s="6" t="n"/>
       <c r="N41" s="6" t="n"/>
       <c r="O41" s="4" t="n"/>
@@ -2600,7 +2734,7 @@
       <c r="I42" s="3" t="n"/>
       <c r="J42" s="3" t="n"/>
       <c r="K42" s="4" t="n"/>
-      <c r="L42" s="29" t="n"/>
+      <c r="L42" s="33" t="n"/>
       <c r="M42" s="6" t="n"/>
       <c r="N42" s="6" t="n"/>
       <c r="O42" s="4" t="n"/>
@@ -2621,7 +2755,7 @@
       <c r="I43" s="3" t="n"/>
       <c r="J43" s="3" t="n"/>
       <c r="K43" s="4" t="n"/>
-      <c r="L43" s="29" t="n"/>
+      <c r="L43" s="33" t="n"/>
       <c r="M43" s="6" t="n"/>
       <c r="N43" s="6" t="n"/>
       <c r="O43" s="4" t="n"/>
@@ -2642,7 +2776,7 @@
       <c r="I44" s="3" t="n"/>
       <c r="J44" s="3" t="n"/>
       <c r="K44" s="4" t="n"/>
-      <c r="L44" s="29" t="n"/>
+      <c r="L44" s="33" t="n"/>
       <c r="M44" s="6" t="n"/>
       <c r="N44" s="6" t="n"/>
       <c r="O44" s="4" t="n"/>
@@ -4334,530 +4468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:S9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14.28515625" customWidth="1" min="1" max="1"/>
-    <col width="14.28515625" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="36.140625" customWidth="1" min="5" max="5"/>
-    <col width="36.140625" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="14.28515625" customWidth="1" min="9" max="9"/>
-    <col width="14.28515625" customWidth="1" min="10" max="10"/>
-    <col width="15" customWidth="1" min="11" max="11"/>
-    <col width="15" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="13" customWidth="1" min="14" max="14"/>
-    <col width="15" customWidth="1" min="15" max="15"/>
-    <col width="13" customWidth="1" min="16" max="16"/>
-    <col width="18" customWidth="1" min="17" max="17"/>
-    <col width="26" customWidth="1" min="18" max="18"/>
-    <col width="14" customWidth="1" min="19" max="19"/>
-  </cols>
-  <sheetData>
-    <row r="2">
-      <c r="A2" s="15" t="inlineStr">
-        <is>
-          <t>Client Count</t>
-        </is>
-      </c>
-      <c r="B2" s="15" t="inlineStr">
-        <is>
-          <t>Owner First Name</t>
-        </is>
-      </c>
-      <c r="C2" s="15" t="inlineStr">
-        <is>
-          <t>Owner Last Name</t>
-        </is>
-      </c>
-      <c r="D2" s="15" t="inlineStr">
-        <is>
-          <t>New Payroll or Existing Payroll this year</t>
-        </is>
-      </c>
-      <c r="E2" s="15" t="inlineStr">
-        <is>
-          <t>Client Legal Name</t>
-        </is>
-      </c>
-      <c r="F2" s="15" t="inlineStr">
-        <is>
-          <t>EIN</t>
-        </is>
-      </c>
-      <c r="G2" s="15" t="inlineStr">
-        <is>
-          <t>Address</t>
-        </is>
-      </c>
-      <c r="H2" s="15" t="inlineStr">
-        <is>
-          <t>City, State Zipcode</t>
-        </is>
-      </c>
-      <c r="I2" s="15" t="inlineStr">
-        <is>
-          <t>Avg # of EEs paid each payroll</t>
-        </is>
-      </c>
-      <c r="J2" s="15" t="inlineStr">
-        <is>
-          <t>Payroll Frequency</t>
-        </is>
-      </c>
-      <c r="K2" s="15" t="inlineStr">
-        <is>
-          <t>Payroll Frequency</t>
-        </is>
-      </c>
-      <c r="L2" s="15" t="inlineStr">
-        <is>
-          <t>Fee Per payroll run</t>
-        </is>
-      </c>
-      <c r="M2" s="15" t="inlineStr">
-        <is>
-          <t>Run Rate</t>
-        </is>
-      </c>
-      <c r="N2" s="15" t="inlineStr">
-        <is>
-          <t>401K Plan</t>
-        </is>
-      </c>
-      <c r="O2" s="15" t="inlineStr">
-        <is>
-          <t>401K Fees</t>
-        </is>
-      </c>
-      <c r="P2" s="15" t="inlineStr">
-        <is>
-          <t>Other CY Fees</t>
-        </is>
-      </c>
-      <c r="Q2" s="15" t="inlineStr">
-        <is>
-          <t>Total Current Annualized Billings (Excluding Year End/W2 Fees)</t>
-        </is>
-      </c>
-      <c r="R2" s="15" t="inlineStr">
-        <is>
-          <t>Payroll Package</t>
-        </is>
-      </c>
-      <c r="S2" s="15" t="inlineStr">
-        <is>
-          <t>Invoice on file</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Oliver</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Beirne</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>B333 Trading Group LLC</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>42-2175878</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>980 N Federal Hwy Suite 314</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Boca Raton FL 33432</t>
-        </is>
-      </c>
-      <c r="I3" t="n">
-        <v>2</v>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Monthly</t>
-        </is>
-      </c>
-      <c r="K3" t="n">
-        <v>12</v>
-      </c>
-      <c r="L3" s="31" t="n">
-        <v>129.6</v>
-      </c>
-      <c r="M3" s="31">
-        <f>K3*L3</f>
-        <v/>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="Q3" s="31">
-        <f>M3</f>
-        <v/>
-      </c>
-      <c r="R3" s="15" t="inlineStr">
-        <is>
-          <t>ADP Enhanced Payroll</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Anthony </t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Gerb </t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>AJG Trading LLC</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>41-5035542</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>1881 N Nash Street Apt No 705</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Arlington, VA 22209</t>
-        </is>
-      </c>
-      <c r="I4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Monthly</t>
-        </is>
-      </c>
-      <c r="K4" t="n">
-        <v>12</v>
-      </c>
-      <c r="L4" s="31" t="n">
-        <v>125.95</v>
-      </c>
-      <c r="M4" s="31">
-        <f>K4*L4</f>
-        <v/>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="Q4" s="31">
-        <f>M4</f>
-        <v/>
-      </c>
-      <c r="R4" s="15" t="inlineStr">
-        <is>
-          <t>ADP Enhanced Payroll</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Alexander </t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Harris</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Kapstone Digital LLC</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>85-3782692</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>936 SW 1st Ave Apt. No. 406</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Miami, FL 33130</t>
-        </is>
-      </c>
-      <c r="I5" t="n">
-        <v>1</v>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Monthly</t>
-        </is>
-      </c>
-      <c r="K5" t="n">
-        <v>12</v>
-      </c>
-      <c r="L5" s="31" t="n">
-        <v>125.95</v>
-      </c>
-      <c r="M5" s="31">
-        <f>K5*L5</f>
-        <v/>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="Q5" s="31">
-        <f>M5</f>
-        <v/>
-      </c>
-      <c r="R5" s="15" t="inlineStr">
-        <is>
-          <t>ADP Enhanced Payroll</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>John</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Ewing</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Atlas Opera, Inc.</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>82-2302400</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>83 Canal Street</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>New York, NY 10002</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
-        <v>1</v>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Monthly</t>
-        </is>
-      </c>
-      <c r="K6" t="n">
-        <v>12</v>
-      </c>
-      <c r="L6" s="31" t="n">
-        <v>125.95</v>
-      </c>
-      <c r="M6" s="31">
-        <f>K6*L6</f>
-        <v/>
-      </c>
-      <c r="Q6" s="31">
-        <f>M6</f>
-        <v/>
-      </c>
-      <c r="R6" s="15" t="inlineStr">
-        <is>
-          <t>ADP Enhanced Payroll</t>
-        </is>
-      </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>5</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Christina </t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pellicane </t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>North Star Works, LLC</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>42-4495054</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>121 S Colts Neck Way</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Hockessin, DE 19707</t>
-        </is>
-      </c>
-      <c r="I7" t="n">
-        <v>1</v>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>Monthly</t>
-        </is>
-      </c>
-      <c r="K7" t="n">
-        <v>12</v>
-      </c>
-      <c r="L7" s="31" t="n">
-        <v>125.95</v>
-      </c>
-      <c r="M7" s="31">
-        <f>K7*L7</f>
-        <v/>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="Q7" s="31">
-        <f>M7</f>
-        <v/>
-      </c>
-      <c r="R7" s="15" t="inlineStr">
-        <is>
-          <t>ADP Enhanced Payroll</t>
-        </is>
-      </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="L9" s="15" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="M9" s="31">
-        <f>SUM(M3:M7)</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -4870,226 +4481,226 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="32" t="inlineStr">
+      <c r="A1" s="46" t="inlineStr">
         <is>
           <t>ADP RUN PAYROLL PACKAGES — ZONE 7 LIST</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="33" t="inlineStr">
-        <is>
-          <t>List price per payroll run. The package is locked at submission. The price can be adjusted.</t>
+      <c r="A2" s="47" t="inlineStr">
+        <is>
+          <t>List price per payroll run. The package is locked at submission. The price is adjustable.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="34" t="inlineStr">
+      <c r="A4" s="48" t="inlineStr">
         <is>
           <t>Package</t>
         </is>
       </c>
-      <c r="B4" s="34" t="inlineStr">
+      <c r="B4" s="48" t="inlineStr">
         <is>
           <t>Weekly</t>
         </is>
       </c>
-      <c r="C4" s="34" t="inlineStr">
+      <c r="C4" s="48" t="inlineStr">
         <is>
           <t>Bi-weekly</t>
         </is>
       </c>
-      <c r="D4" s="34" t="inlineStr">
+      <c r="D4" s="48" t="inlineStr">
         <is>
           <t>Semi-monthly</t>
         </is>
       </c>
-      <c r="E4" s="34" t="inlineStr">
+      <c r="E4" s="48" t="inlineStr">
         <is>
           <t>Monthly</t>
         </is>
       </c>
-      <c r="F4" s="34" t="inlineStr">
+      <c r="F4" s="48" t="inlineStr">
         <is>
           <t>Quarterly</t>
         </is>
       </c>
-      <c r="G4" s="34" t="inlineStr">
+      <c r="G4" s="48" t="inlineStr">
         <is>
           <t>Annual</t>
         </is>
       </c>
     </row>
     <row r="5" ht="52" customHeight="1">
-      <c r="A5" s="35" t="inlineStr">
+      <c r="A5" s="49" t="inlineStr">
         <is>
           <t>ADP Essential Payroll</t>
         </is>
       </c>
-      <c r="B5" s="36" t="inlineStr">
+      <c r="B5" s="50" t="inlineStr">
         <is>
           <t>$40.95 ees 1-2
 $46.95 ees 3-4
 +$2.75 over 4</t>
         </is>
       </c>
-      <c r="C5" s="36" t="inlineStr">
+      <c r="C5" s="50" t="inlineStr">
         <is>
           <t>$65.95 ees 1-2
 $71.95 ees 3-4
 +$2.70 over 4</t>
         </is>
       </c>
-      <c r="D5" s="36" t="inlineStr">
+      <c r="D5" s="50" t="inlineStr">
         <is>
           <t>$69.95 ees 1-2
 $75.95 ees 3-4
 +$2.95 over 4</t>
         </is>
       </c>
-      <c r="E5" s="36" t="inlineStr">
+      <c r="E5" s="50" t="inlineStr">
         <is>
           <t>$79 base
 +$4 per employee</t>
         </is>
       </c>
-      <c r="F5" s="36" t="inlineStr">
+      <c r="F5" s="50" t="inlineStr">
         <is>
           <t>$127.95</t>
         </is>
       </c>
-      <c r="G5" s="36" t="inlineStr">
+      <c r="G5" s="50" t="inlineStr">
         <is>
           <t>$500.00</t>
         </is>
       </c>
     </row>
     <row r="6" ht="52" customHeight="1">
-      <c r="A6" s="35" t="inlineStr">
+      <c r="A6" s="49" t="inlineStr">
         <is>
           <t>ADP Enhanced Payroll</t>
         </is>
       </c>
-      <c r="B6" s="36" t="inlineStr">
+      <c r="B6" s="50" t="inlineStr">
         <is>
           <t>$64.50 base
 +$3.15 each over 1</t>
         </is>
       </c>
-      <c r="C6" s="36" t="inlineStr">
+      <c r="C6" s="50" t="inlineStr">
         <is>
           <t>$92.95 base
 +$3.60 each over 1</t>
         </is>
       </c>
-      <c r="D6" s="36" t="inlineStr">
+      <c r="D6" s="50" t="inlineStr">
         <is>
           <t>$98.95 base
 +$3.80 each over 1</t>
         </is>
       </c>
-      <c r="E6" s="36" t="inlineStr">
+      <c r="E6" s="50" t="inlineStr">
         <is>
           <t>$125.95 base
 +$3.65 each over 1</t>
         </is>
       </c>
-      <c r="F6" s="36" t="inlineStr">
+      <c r="F6" s="50" t="inlineStr">
         <is>
           <t>$199.95</t>
         </is>
       </c>
-      <c r="G6" s="36" t="inlineStr">
+      <c r="G6" s="50" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="7" ht="52" customHeight="1">
-      <c r="A7" s="35" t="inlineStr">
+      <c r="A7" s="49" t="inlineStr">
         <is>
           <t>ADP Complete Payroll and HR Plus</t>
         </is>
       </c>
-      <c r="B7" s="36" t="inlineStr">
+      <c r="B7" s="50" t="inlineStr">
         <is>
           <t>$92.95 ees 1-2
 $98.95 ees 3-4
 +$3.40 over 4</t>
         </is>
       </c>
-      <c r="C7" s="36" t="inlineStr">
+      <c r="C7" s="50" t="inlineStr">
         <is>
           <t>$169.95 ees 1-2
 $175.95 ees 3-4
 +$4.75 over 4</t>
         </is>
       </c>
-      <c r="D7" s="36" t="inlineStr">
+      <c r="D7" s="50" t="inlineStr">
         <is>
           <t>$181.95 ees 1-2
 $188.95 ees 3-4
 +$4.80 over 4</t>
         </is>
       </c>
-      <c r="E7" s="36" t="inlineStr">
+      <c r="E7" s="50" t="inlineStr">
         <is>
           <t>$258.95 ees 1-2
 $264.95 ees 3-4
 +$4.30 over 4</t>
         </is>
       </c>
-      <c r="F7" s="36" t="inlineStr">
+      <c r="F7" s="50" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G7" s="36" t="inlineStr">
+      <c r="G7" s="50" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="8" ht="52" customHeight="1">
-      <c r="A8" s="35" t="inlineStr">
+      <c r="A8" s="49" t="inlineStr">
         <is>
           <t>ADP HR Pro</t>
         </is>
       </c>
-      <c r="B8" s="36" t="inlineStr">
+      <c r="B8" s="50" t="inlineStr">
         <is>
           <t>$132.95 ees 1-2
 $139.95 ees 3-4
 +$4.25 over 4</t>
         </is>
       </c>
-      <c r="C8" s="36" t="inlineStr">
+      <c r="C8" s="50" t="inlineStr">
         <is>
           <t>$254.95 ees 1-2
 $261.95 ees 3-4
 +$5.00 over 4</t>
         </is>
       </c>
-      <c r="D8" s="36" t="inlineStr">
+      <c r="D8" s="50" t="inlineStr">
         <is>
           <t>$269.95 ees 1-2
 $276.95 ees 3-4
 +$5.05 over 4</t>
         </is>
       </c>
-      <c r="E8" s="36" t="inlineStr">
+      <c r="E8" s="50" t="inlineStr">
         <is>
           <t>$399.95 ees 1-2
 $406.95 ees 3-4
 +$4.90 over 4</t>
         </is>
       </c>
-      <c r="F8" s="36" t="inlineStr">
+      <c r="F8" s="50" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G8" s="36" t="inlineStr">
+      <c r="G8" s="50" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -5112,7 +4723,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Walters Mirrors — HR Pro. Bi-weekly, 3 employees, 261.95.</t>
+          <t xml:space="preserve">   Walters Mirrors — HR Pro, bi-weekly, 3 employees. List 261.95.</t>
         </is>
       </c>
     </row>
@@ -5127,17 +4738,38 @@
       <c r="A14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Prices above are list with no discount applied.</t>
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>TWO PRICES SIT ABOVE ENHANCED LIST — shaded amber on Sheet1</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Wisdom by Woods, 129.78 against 125.95 list.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Auction Time Pieces, 154.10 against 102.75 list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Either cap them at list or move them to Complete, which lists at 258.95 and 181.95.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>Source: FY25 SBS RUN Price Book, Zone 7, 2nd Release. ADP internal.</t>
         </is>

</xml_diff>

<commit_message>
Move Wisdom and Auction to Complete package
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HvXhTSq2hCmheT3mKtqmHP
</commit_message>
<xml_diff>
--- a/output/stephen/CBA_Innovative_Advisors_ADP_2026-09-24.xlsx
+++ b/output/stephen/CBA_Innovative_Advisors_ADP_2026-09-24.xlsx
@@ -1173,7 +1173,7 @@
       <c r="K7" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="L7" s="27" t="n">
+      <c r="L7" s="28" t="n">
         <v>129.78</v>
       </c>
       <c r="M7" s="28">
@@ -1189,11 +1189,11 @@
       </c>
       <c r="R7" s="15" t="inlineStr">
         <is>
-          <t>ADP Enhanced Payroll</t>
-        </is>
-      </c>
-      <c r="S7" s="31" t="n">
-        <v>125.95</v>
+          <t>ADP Complete Payroll and HR Plus</t>
+        </is>
+      </c>
+      <c r="S7" s="32" t="n">
+        <v>258.95</v>
       </c>
       <c r="T7" t="inlineStr">
         <is>
@@ -1251,7 +1251,7 @@
       <c r="K8" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="L8" s="27" t="n">
+      <c r="L8" s="28" t="n">
         <v>154.1</v>
       </c>
       <c r="M8" s="28">
@@ -1267,11 +1267,11 @@
       </c>
       <c r="R8" s="15" t="inlineStr">
         <is>
-          <t>ADP Enhanced Payroll</t>
-        </is>
-      </c>
-      <c r="S8" s="31" t="n">
-        <v>102.75</v>
+          <t>ADP Complete Payroll and HR Plus</t>
+        </is>
+      </c>
+      <c r="S8" s="32" t="n">
+        <v>181.95</v>
       </c>
       <c r="T8" t="inlineStr">
         <is>
@@ -4468,7 +4468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -4716,7 +4716,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Everyone is on Enhanced except two.</t>
+          <t xml:space="preserve">   Everyone is on Enhanced except four.</t>
         </is>
       </c>
     </row>
@@ -4735,12 +4735,16 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr"/>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Wisdom by Woods and Auction Time Pieces — Complete. Both price above Enhanced list, so Complete is the right fit.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>TWO PRICES SIT ABOVE ENHANCED LIST — shaded amber on Sheet1</t>
+          <t xml:space="preserve">   Wisdom 129.78 against Complete list 258.95. Auction 154.10 against Complete list 181.95. Both now sit under list.</t>
         </is>
       </c>
     </row>
@@ -4765,9 +4769,7 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr"/>
-    </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
@@ -4775,6 +4777,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>

</xml_diff>